<commit_message>
Actualización de datos Balanz cierre 21-09-26
</commit_message>
<xml_diff>
--- a/mi_cartera_balanz/data/Reporte_Avanzado_Cartera.xlsx
+++ b/mi_cartera_balanz/data/Reporte_Avanzado_Cartera.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2497" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2503" uniqueCount="356">
   <si>
     <t>Descripcion</t>
   </si>
@@ -1037,6 +1037,9 @@
   </si>
   <si>
     <t>2026-09-18</t>
+  </si>
+  <si>
+    <t>2026-09-21</t>
   </si>
   <si>
     <t>2024-04-11</t>
@@ -4432,7 +4435,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -4478,90 +4481,64 @@
         <v>190</v>
       </c>
       <c r="F2">
-        <v>8770</v>
+        <v>8500</v>
       </c>
       <c r="G2">
-        <v>877000</v>
+        <v>850000</v>
       </c>
       <c r="H2">
-        <v>150329.3307692307</v>
+        <v>123329.3307692307</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>200</v>
       </c>
       <c r="B3">
-        <v>139</v>
+        <v>42</v>
       </c>
       <c r="C3">
-        <v>14258.8864028777</v>
+        <v>24183.39547619048</v>
       </c>
       <c r="D3">
-        <v>1981985.21</v>
+        <v>1015702.61</v>
       </c>
       <c r="E3" t="s">
         <v>190</v>
       </c>
       <c r="F3">
-        <v>14810</v>
+        <v>24220</v>
       </c>
       <c r="G3">
-        <v>2058590</v>
+        <v>1017240</v>
       </c>
       <c r="H3">
-        <v>76604.79000000004</v>
+        <v>1537.390000000014</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B4">
-        <v>42</v>
+        <v>160170.68</v>
       </c>
       <c r="C4">
-        <v>24183.39547619048</v>
+        <v>12.48667983428678</v>
       </c>
       <c r="D4">
-        <v>1015702.61</v>
+        <v>2000000</v>
       </c>
       <c r="E4" t="s">
         <v>190</v>
       </c>
       <c r="F4">
-        <v>23780</v>
+        <v>12.505889</v>
       </c>
       <c r="G4">
-        <v>998760</v>
+        <v>2003076.74513452</v>
       </c>
       <c r="H4">
-        <v>-16942.60999999999</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>201</v>
-      </c>
-      <c r="B5">
-        <v>160170.68</v>
-      </c>
-      <c r="C5">
-        <v>12.48667983428678</v>
-      </c>
-      <c r="D5">
-        <v>2000000</v>
-      </c>
-      <c r="E5" t="s">
-        <v>190</v>
-      </c>
-      <c r="F5">
-        <v>12.505889</v>
-      </c>
-      <c r="G5">
-        <v>2003076.74513452</v>
-      </c>
-      <c r="H5">
         <v>3076.745134519879</v>
       </c>
     </row>
@@ -4572,7 +4549,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -8733,6 +8710,32 @@
       </c>
       <c r="H160">
         <v>51530.33423076922</v>
+      </c>
+    </row>
+    <row r="161" spans="1:8">
+      <c r="A161" s="1">
+        <v>46279</v>
+      </c>
+      <c r="B161" s="1">
+        <v>46286</v>
+      </c>
+      <c r="C161" t="s">
+        <v>83</v>
+      </c>
+      <c r="D161" t="s">
+        <v>190</v>
+      </c>
+      <c r="E161">
+        <v>139</v>
+      </c>
+      <c r="F161">
+        <v>14258.8864028777</v>
+      </c>
+      <c r="G161">
+        <v>15034.24086330935</v>
+      </c>
+      <c r="H161">
+        <v>107774.2700000001</v>
       </c>
     </row>
   </sheetData>
@@ -8742,7 +8745,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -8799,79 +8802,53 @@
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>200</v>
       </c>
       <c r="B3" s="1">
-        <v>46279</v>
+        <v>46283</v>
       </c>
       <c r="C3">
-        <v>139</v>
+        <v>42</v>
       </c>
       <c r="D3">
-        <v>14080</v>
+        <v>23880</v>
       </c>
       <c r="E3">
-        <v>178.886402877697</v>
+        <v>303.3954761904752</v>
       </c>
       <c r="F3">
-        <v>14258.8864028777</v>
+        <v>24183.39547619048</v>
       </c>
       <c r="G3">
-        <v>14442.37680311301</v>
+        <v>24494.59944022999</v>
       </c>
       <c r="H3">
-        <v>1981985.21</v>
+        <v>1015702.61</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B4" s="1">
-        <v>46283</v>
+        <v>46286.80225602954</v>
       </c>
       <c r="C4">
-        <v>42</v>
+        <v>160170.68</v>
       </c>
       <c r="D4">
-        <v>23880</v>
+        <v>12.48667983428678</v>
       </c>
       <c r="E4">
-        <v>303.3954761904752</v>
+        <v>0</v>
       </c>
       <c r="F4">
-        <v>24183.39547619048</v>
+        <v>12.48667983428678</v>
       </c>
       <c r="G4">
-        <v>24494.59944022999</v>
+        <v>12.48667983428678</v>
       </c>
       <c r="H4">
-        <v>1015702.61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" t="s">
-        <v>201</v>
-      </c>
-      <c r="B5" s="1">
-        <v>46285.60431405393</v>
-      </c>
-      <c r="C5">
-        <v>160170.68</v>
-      </c>
-      <c r="D5">
-        <v>12.48667983428678</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>12.48667983428678</v>
-      </c>
-      <c r="G5">
-        <v>12.48667983428678</v>
-      </c>
-      <c r="H5">
         <v>2000000</v>
       </c>
     </row>
@@ -8898,7 +8875,7 @@
         <v>242</v>
       </c>
       <c r="B2">
-        <v>536974.775</v>
+        <v>549702.525</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -8906,7 +8883,7 @@
         <v>243</v>
       </c>
       <c r="B3">
-        <v>43413.71000000001</v>
+        <v>44686.48</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -8914,7 +8891,7 @@
         <v>244</v>
       </c>
       <c r="B4">
-        <v>580388.485</v>
+        <v>594389.005</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -8996,7 +8973,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P219"/>
+  <dimension ref="A1:P220"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
@@ -9666,7 +9643,7 @@
         <v>287</v>
       </c>
       <c r="F14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G14">
         <v>26</v>
@@ -9716,7 +9693,7 @@
         <v>287</v>
       </c>
       <c r="F15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -9766,7 +9743,7 @@
         <v>287</v>
       </c>
       <c r="F16" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -9816,7 +9793,7 @@
         <v>287</v>
       </c>
       <c r="F17" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G17">
         <v>3</v>
@@ -9866,7 +9843,7 @@
         <v>288</v>
       </c>
       <c r="F18" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G18">
         <v>55</v>
@@ -9916,7 +9893,7 @@
         <v>289</v>
       </c>
       <c r="F19" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G19">
         <v>6</v>
@@ -9966,7 +9943,7 @@
         <v>289</v>
       </c>
       <c r="F20" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G20">
         <v>4</v>
@@ -10016,7 +9993,7 @@
         <v>289</v>
       </c>
       <c r="F21" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G21">
         <v>5</v>
@@ -10066,7 +10043,7 @@
         <v>289</v>
       </c>
       <c r="F22" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G22">
         <v>4</v>
@@ -10116,7 +10093,7 @@
         <v>289</v>
       </c>
       <c r="F23" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -10166,7 +10143,7 @@
         <v>289</v>
       </c>
       <c r="F24" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G24">
         <v>4</v>
@@ -10216,7 +10193,7 @@
         <v>289</v>
       </c>
       <c r="F25" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G25">
         <v>5</v>
@@ -10266,7 +10243,7 @@
         <v>290</v>
       </c>
       <c r="F26" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G26">
         <v>9</v>
@@ -10316,7 +10293,7 @@
         <v>290</v>
       </c>
       <c r="F27" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G27">
         <v>6</v>
@@ -10366,7 +10343,7 @@
         <v>290</v>
       </c>
       <c r="F28" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G28">
         <v>5</v>
@@ -10416,7 +10393,7 @@
         <v>290</v>
       </c>
       <c r="F29" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G29">
         <v>2</v>
@@ -10466,7 +10443,7 @@
         <v>290</v>
       </c>
       <c r="F30" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G30">
         <v>2</v>
@@ -10516,7 +10493,7 @@
         <v>290</v>
       </c>
       <c r="F31" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G31">
         <v>7</v>
@@ -10716,7 +10693,7 @@
         <v>293</v>
       </c>
       <c r="F35" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G35">
         <v>5</v>
@@ -10766,7 +10743,7 @@
         <v>293</v>
       </c>
       <c r="F36" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G36">
         <v>10</v>
@@ -10816,7 +10793,7 @@
         <v>293</v>
       </c>
       <c r="F37" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G37">
         <v>2</v>
@@ -10866,7 +10843,7 @@
         <v>293</v>
       </c>
       <c r="F38" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G38">
         <v>16</v>
@@ -10916,7 +10893,7 @@
         <v>293</v>
       </c>
       <c r="F39" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G39">
         <v>10</v>
@@ -10966,7 +10943,7 @@
         <v>293</v>
       </c>
       <c r="F40" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G40">
         <v>1</v>
@@ -11016,7 +10993,7 @@
         <v>294</v>
       </c>
       <c r="F41" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G41">
         <v>9</v>
@@ -11066,7 +11043,7 @@
         <v>294</v>
       </c>
       <c r="F42" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G42">
         <v>100</v>
@@ -11116,7 +11093,7 @@
         <v>294</v>
       </c>
       <c r="F43" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G43">
         <v>21</v>
@@ -12016,7 +11993,7 @@
         <v>296</v>
       </c>
       <c r="F61" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G61">
         <v>4</v>
@@ -12916,7 +12893,7 @@
         <v>298</v>
       </c>
       <c r="F79" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G79">
         <v>5</v>
@@ -13966,7 +13943,7 @@
         <v>305</v>
       </c>
       <c r="F100" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G100">
         <v>297</v>
@@ -14966,7 +14943,7 @@
         <v>310</v>
       </c>
       <c r="F120" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G120">
         <v>100</v>
@@ -16066,7 +16043,7 @@
         <v>312</v>
       </c>
       <c r="F142" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G142">
         <v>33</v>
@@ -19066,7 +19043,7 @@
         <v>328</v>
       </c>
       <c r="F202" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G202">
         <v>90</v>
@@ -19866,7 +19843,7 @@
         <v>337</v>
       </c>
       <c r="F218" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G218">
         <v>100</v>
@@ -19947,6 +19924,56 @@
       </c>
       <c r="P219">
         <v>23880</v>
+      </c>
+    </row>
+    <row r="220" spans="1:16">
+      <c r="A220" t="s">
+        <v>265</v>
+      </c>
+      <c r="B220">
+        <v>10641020</v>
+      </c>
+      <c r="C220" t="s">
+        <v>83</v>
+      </c>
+      <c r="D220" t="s">
+        <v>285</v>
+      </c>
+      <c r="E220" t="s">
+        <v>339</v>
+      </c>
+      <c r="F220" t="s">
+        <v>339</v>
+      </c>
+      <c r="G220">
+        <v>139</v>
+      </c>
+      <c r="H220">
+        <v>15134.9640287769</v>
+      </c>
+      <c r="I220">
+        <v>2103760</v>
+      </c>
+      <c r="J220">
+        <v>1272.77</v>
+      </c>
+      <c r="K220">
+        <v>12727.75</v>
+      </c>
+      <c r="L220">
+        <v>2089759.48</v>
+      </c>
+      <c r="M220" t="s">
+        <v>190</v>
+      </c>
+      <c r="N220" s="1">
+        <v>46286</v>
+      </c>
+      <c r="O220" t="s">
+        <v>83</v>
+      </c>
+      <c r="P220">
+        <v>15134.9640287769</v>
       </c>
     </row>
   </sheetData>
@@ -19969,7 +19996,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B2">
         <v>1000000</v>
@@ -19977,18 +20004,18 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B3">
-        <v>1184719.876087911</v>
+        <v>1292494.146087911</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B4">
-        <v>1213068.255903751</v>
+        <v>1127943.465903751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agrega tarjeta de Techo de Recompra en Reportes
</commit_message>
<xml_diff>
--- a/mi_cartera_balanz/data/Reporte_Avanzado_Cartera.xlsx
+++ b/mi_cartera_balanz/data/Reporte_Avanzado_Cartera.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2510" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2520" uniqueCount="359">
   <si>
     <t>Descripcion</t>
   </si>
@@ -622,6 +622,9 @@
     <t>Ganancia/Perdida NO Realizada ($)</t>
   </si>
   <si>
+    <t>PAMPA ENERGIA</t>
+  </si>
+  <si>
     <t>MELI</t>
   </si>
   <si>
@@ -652,9 +655,6 @@
     <t>CEDEAR BROADCOM INC.</t>
   </si>
   <si>
-    <t>PAMPA ENERGIA</t>
-  </si>
-  <si>
     <t>GRUPO FINANCIERO GALICIA "B"1V.ESC.</t>
   </si>
   <si>
@@ -1042,6 +1042,9 @@
     <t>2026-09-21</t>
   </si>
   <si>
+    <t>2026-09-24</t>
+  </si>
+  <si>
     <t>2024-04-11</t>
   </si>
   <si>
@@ -1082,6 +1085,9 @@
   </si>
   <si>
     <t>2026-09-22</t>
+  </si>
+  <si>
+    <t>2026-09-25</t>
   </si>
   <si>
     <t>Flujo Fondeo Neto</t>
@@ -4438,7 +4444,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -4469,54 +4475,54 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>200</v>
       </c>
       <c r="B2">
-        <v>332</v>
+        <v>195</v>
       </c>
       <c r="C2">
-        <v>8192.675810936051</v>
+        <v>5144.007025641025</v>
       </c>
       <c r="D2">
-        <v>2719968.369230769</v>
+        <v>1003081.37</v>
       </c>
       <c r="E2" t="s">
         <v>190</v>
       </c>
       <c r="F2">
-        <v>8500</v>
+        <v>5110</v>
       </c>
       <c r="G2">
-        <v>2822000</v>
+        <v>996450</v>
       </c>
       <c r="H2">
-        <v>102031.6307692309</v>
+        <v>-6631.369999999995</v>
       </c>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" t="s">
-        <v>200</v>
+        <v>82</v>
       </c>
       <c r="B3">
-        <v>42</v>
+        <v>332</v>
       </c>
       <c r="C3">
-        <v>24183.39547619048</v>
+        <v>8192.675810936051</v>
       </c>
       <c r="D3">
-        <v>1015702.61</v>
+        <v>2719968.369230769</v>
       </c>
       <c r="E3" t="s">
         <v>190</v>
       </c>
       <c r="F3">
-        <v>24220</v>
+        <v>8450</v>
       </c>
       <c r="G3">
-        <v>1017240</v>
+        <v>2805400</v>
       </c>
       <c r="H3">
-        <v>1537.390000000014</v>
+        <v>85431.63076923089</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -4524,24 +4530,50 @@
         <v>201</v>
       </c>
       <c r="B4">
-        <v>2113593.05</v>
+        <v>42</v>
       </c>
       <c r="C4">
+        <v>24183.39547619048</v>
+      </c>
+      <c r="D4">
+        <v>1015702.61</v>
+      </c>
+      <c r="E4" t="s">
+        <v>190</v>
+      </c>
+      <c r="F4">
+        <v>23670</v>
+      </c>
+      <c r="G4">
+        <v>994140</v>
+      </c>
+      <c r="H4">
+        <v>-21562.60999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>202</v>
+      </c>
+      <c r="B5">
+        <v>1110511.68</v>
+      </c>
+      <c r="C5">
         <v>1</v>
       </c>
-      <c r="D4">
-        <v>2113593.05</v>
-      </c>
-      <c r="E4" t="s">
-        <v>190</v>
-      </c>
-      <c r="F4">
+      <c r="D5">
+        <v>1110511.68</v>
+      </c>
+      <c r="E5" t="s">
+        <v>190</v>
+      </c>
+      <c r="F5">
         <v>1</v>
       </c>
-      <c r="G4">
-        <v>2113593.05</v>
-      </c>
-      <c r="H4">
+      <c r="G5">
+        <v>1110511.68</v>
+      </c>
+      <c r="H5">
         <v>0</v>
       </c>
     </row>
@@ -4557,10 +4589,10 @@
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -4572,13 +4604,13 @@
         <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="2" spans="1:8">
@@ -4589,7 +4621,7 @@
         <v>45391</v>
       </c>
       <c r="C2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D2" t="s">
         <v>190</v>
@@ -4615,7 +4647,7 @@
         <v>45391</v>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D3" t="s">
         <v>190</v>
@@ -4641,7 +4673,7 @@
         <v>45391</v>
       </c>
       <c r="C4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D4" t="s">
         <v>190</v>
@@ -4667,7 +4699,7 @@
         <v>45414</v>
       </c>
       <c r="C5" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D5" t="s">
         <v>190</v>
@@ -4849,7 +4881,7 @@
         <v>45419</v>
       </c>
       <c r="C12" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D12" t="s">
         <v>190</v>
@@ -5057,7 +5089,7 @@
         <v>45443</v>
       </c>
       <c r="C20" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D20" t="s">
         <v>190</v>
@@ -5187,7 +5219,7 @@
         <v>45481</v>
       </c>
       <c r="C25" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D25" t="s">
         <v>190</v>
@@ -5265,7 +5297,7 @@
         <v>45509</v>
       </c>
       <c r="C28" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D28" t="s">
         <v>190</v>
@@ -5733,7 +5765,7 @@
         <v>45583</v>
       </c>
       <c r="C46" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D46" t="s">
         <v>190</v>
@@ -5759,7 +5791,7 @@
         <v>45583</v>
       </c>
       <c r="C47" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D47" t="s">
         <v>190</v>
@@ -6773,7 +6805,7 @@
         <v>45674</v>
       </c>
       <c r="C86" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D86" t="s">
         <v>190</v>
@@ -7189,7 +7221,7 @@
         <v>45852</v>
       </c>
       <c r="C102" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D102" t="s">
         <v>190</v>
@@ -7215,7 +7247,7 @@
         <v>45852</v>
       </c>
       <c r="C103" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D103" t="s">
         <v>190</v>
@@ -7241,7 +7273,7 @@
         <v>45852</v>
       </c>
       <c r="C104" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D104" t="s">
         <v>190</v>
@@ -8748,7 +8780,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -8779,28 +8811,28 @@
     </row>
     <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>82</v>
+        <v>200</v>
       </c>
       <c r="B2" s="1">
-        <v>46197</v>
+        <v>46289</v>
       </c>
       <c r="C2">
-        <v>100</v>
+        <v>195</v>
       </c>
       <c r="D2">
-        <v>7210</v>
+        <v>5110</v>
       </c>
       <c r="E2">
-        <v>56.70669230769272</v>
+        <v>34.00702564102539</v>
       </c>
       <c r="F2">
-        <v>7266.706692307693</v>
+        <v>5144.007025641025</v>
       </c>
       <c r="G2">
-        <v>7324.312452726859</v>
+        <v>5178.469716921776</v>
       </c>
       <c r="H2">
-        <v>726670.6692307693</v>
+        <v>1003081.37</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -8808,50 +8840,76 @@
         <v>82</v>
       </c>
       <c r="B3" s="1">
-        <v>46286</v>
+        <v>46197</v>
       </c>
       <c r="C3">
-        <v>232</v>
+        <v>100</v>
       </c>
       <c r="D3">
-        <v>8535</v>
+        <v>7210</v>
       </c>
       <c r="E3">
-        <v>56.80043103448224</v>
+        <v>56.70669230769272</v>
       </c>
       <c r="F3">
-        <v>8591.800431034482</v>
+        <v>7266.706692307693</v>
       </c>
       <c r="G3">
-        <v>8649.361940866287</v>
+        <v>7324.312452726859</v>
       </c>
       <c r="H3">
-        <v>1993297.7</v>
+        <v>726670.6692307693</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>200</v>
+        <v>82</v>
       </c>
       <c r="B4" s="1">
+        <v>46286</v>
+      </c>
+      <c r="C4">
+        <v>232</v>
+      </c>
+      <c r="D4">
+        <v>8535</v>
+      </c>
+      <c r="E4">
+        <v>56.80043103448224</v>
+      </c>
+      <c r="F4">
+        <v>8591.800431034482</v>
+      </c>
+      <c r="G4">
+        <v>8649.361940866287</v>
+      </c>
+      <c r="H4">
+        <v>1993297.7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B5" s="1">
         <v>46283</v>
       </c>
-      <c r="C4">
+      <c r="C5">
         <v>42</v>
       </c>
-      <c r="D4">
+      <c r="D5">
         <v>23880</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <v>303.3954761904752</v>
       </c>
-      <c r="F4">
+      <c r="F5">
         <v>24183.39547619048</v>
       </c>
-      <c r="G4">
+      <c r="G5">
         <v>24494.59944022999</v>
       </c>
-      <c r="H4">
+      <c r="H5">
         <v>1015702.61</v>
       </c>
     </row>
@@ -8878,7 +8936,7 @@
         <v>242</v>
       </c>
       <c r="B2">
-        <v>561682.255</v>
+        <v>567710.775</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -8886,7 +8944,7 @@
         <v>243</v>
       </c>
       <c r="B3">
-        <v>45884.45</v>
+        <v>46487.3</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -8894,7 +8952,7 @@
         <v>244</v>
       </c>
       <c r="B4">
-        <v>607566.705</v>
+        <v>614198.0750000001</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -8976,7 +9034,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P221"/>
+  <dimension ref="A1:P222"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
@@ -9031,7 +9089,7 @@
     </row>
     <row r="2" spans="1:16">
       <c r="A2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B2">
         <v>2908424</v>
@@ -9073,7 +9131,7 @@
         <v>45390</v>
       </c>
       <c r="O2" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P2">
         <v>1960.05</v>
@@ -9281,7 +9339,7 @@
     </row>
     <row r="7" spans="1:16">
       <c r="A7" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B7">
         <v>2908429</v>
@@ -9323,7 +9381,7 @@
         <v>45390</v>
       </c>
       <c r="O7" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P7">
         <v>16369.5</v>
@@ -9331,7 +9389,7 @@
     </row>
     <row r="8" spans="1:16">
       <c r="A8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B8">
         <v>2908430</v>
@@ -9373,7 +9431,7 @@
         <v>45390</v>
       </c>
       <c r="O8" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="P8">
         <v>35260</v>
@@ -9581,7 +9639,7 @@
     </row>
     <row r="13" spans="1:16">
       <c r="A13" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B13">
         <v>2908435</v>
@@ -9623,7 +9681,7 @@
         <v>45390</v>
       </c>
       <c r="O13" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="P13">
         <v>35634.5</v>
@@ -9646,7 +9704,7 @@
         <v>287</v>
       </c>
       <c r="F14" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G14">
         <v>26</v>
@@ -9681,7 +9739,7 @@
     </row>
     <row r="15" spans="1:16">
       <c r="A15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B15">
         <v>2967527</v>
@@ -9696,7 +9754,7 @@
         <v>287</v>
       </c>
       <c r="F15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G15">
         <v>1</v>
@@ -9723,7 +9781,7 @@
         <v>45391</v>
       </c>
       <c r="O15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P15">
         <v>16524.5</v>
@@ -9731,7 +9789,7 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B16">
         <v>2967528</v>
@@ -9746,7 +9804,7 @@
         <v>287</v>
       </c>
       <c r="F16" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G16">
         <v>1</v>
@@ -9773,7 +9831,7 @@
         <v>45391</v>
       </c>
       <c r="O16" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="P16">
         <v>35645.5</v>
@@ -9781,7 +9839,7 @@
     </row>
     <row r="17" spans="1:16">
       <c r="A17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B17">
         <v>2967529</v>
@@ -9796,7 +9854,7 @@
         <v>287</v>
       </c>
       <c r="F17" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G17">
         <v>3</v>
@@ -9823,7 +9881,7 @@
         <v>45391</v>
       </c>
       <c r="O17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="P17">
         <v>35279.5</v>
@@ -9846,7 +9904,7 @@
         <v>288</v>
       </c>
       <c r="F18" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G18">
         <v>55</v>
@@ -9881,7 +9939,7 @@
     </row>
     <row r="19" spans="1:16">
       <c r="A19" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B19">
         <v>3611569</v>
@@ -9896,7 +9954,7 @@
         <v>289</v>
       </c>
       <c r="F19" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G19">
         <v>6</v>
@@ -9923,7 +9981,7 @@
         <v>45414</v>
       </c>
       <c r="O19" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P19">
         <v>2087</v>
@@ -9946,7 +10004,7 @@
         <v>289</v>
       </c>
       <c r="F20" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G20">
         <v>4</v>
@@ -9996,7 +10054,7 @@
         <v>289</v>
       </c>
       <c r="F21" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G21">
         <v>5</v>
@@ -10046,7 +10104,7 @@
         <v>289</v>
       </c>
       <c r="F22" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G22">
         <v>4</v>
@@ -10096,7 +10154,7 @@
         <v>289</v>
       </c>
       <c r="F23" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G23">
         <v>1</v>
@@ -10146,7 +10204,7 @@
         <v>289</v>
       </c>
       <c r="F24" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G24">
         <v>4</v>
@@ -10196,7 +10254,7 @@
         <v>289</v>
       </c>
       <c r="F25" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G25">
         <v>5</v>
@@ -10231,7 +10289,7 @@
     </row>
     <row r="26" spans="1:16">
       <c r="A26" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B26">
         <v>3771670</v>
@@ -10246,7 +10304,7 @@
         <v>290</v>
       </c>
       <c r="F26" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G26">
         <v>9</v>
@@ -10273,7 +10331,7 @@
         <v>45419</v>
       </c>
       <c r="O26" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P26">
         <v>2177</v>
@@ -10296,7 +10354,7 @@
         <v>290</v>
       </c>
       <c r="F27" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G27">
         <v>6</v>
@@ -10346,7 +10404,7 @@
         <v>290</v>
       </c>
       <c r="F28" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G28">
         <v>5</v>
@@ -10396,7 +10454,7 @@
         <v>290</v>
       </c>
       <c r="F29" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G29">
         <v>2</v>
@@ -10446,7 +10504,7 @@
         <v>290</v>
       </c>
       <c r="F30" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G30">
         <v>2</v>
@@ -10496,7 +10554,7 @@
         <v>290</v>
       </c>
       <c r="F31" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="G31">
         <v>7</v>
@@ -10696,7 +10754,7 @@
         <v>293</v>
       </c>
       <c r="F35" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G35">
         <v>5</v>
@@ -10746,7 +10804,7 @@
         <v>293</v>
       </c>
       <c r="F36" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G36">
         <v>10</v>
@@ -10796,7 +10854,7 @@
         <v>293</v>
       </c>
       <c r="F37" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G37">
         <v>2</v>
@@ -10831,7 +10889,7 @@
     </row>
     <row r="38" spans="1:16">
       <c r="A38" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B38">
         <v>4513894</v>
@@ -10846,7 +10904,7 @@
         <v>293</v>
       </c>
       <c r="F38" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G38">
         <v>16</v>
@@ -10873,7 +10931,7 @@
         <v>45443</v>
       </c>
       <c r="O38" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P38">
         <v>2426</v>
@@ -10896,7 +10954,7 @@
         <v>293</v>
       </c>
       <c r="F39" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G39">
         <v>10</v>
@@ -10946,7 +11004,7 @@
         <v>293</v>
       </c>
       <c r="F40" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="G40">
         <v>1</v>
@@ -10996,7 +11054,7 @@
         <v>294</v>
       </c>
       <c r="F41" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G41">
         <v>9</v>
@@ -11046,7 +11104,7 @@
         <v>294</v>
       </c>
       <c r="F42" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G42">
         <v>100</v>
@@ -11096,7 +11154,7 @@
         <v>294</v>
       </c>
       <c r="F43" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G43">
         <v>21</v>
@@ -11231,7 +11289,7 @@
     </row>
     <row r="46" spans="1:16">
       <c r="A46" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B46">
         <v>5734647</v>
@@ -11273,7 +11331,7 @@
         <v>45481</v>
       </c>
       <c r="O46" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P46">
         <v>2545.3</v>
@@ -11431,7 +11489,7 @@
     </row>
     <row r="50" spans="1:16">
       <c r="A50" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B50">
         <v>6763852</v>
@@ -11473,7 +11531,7 @@
         <v>45509</v>
       </c>
       <c r="O50" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P50">
         <v>2120</v>
@@ -11996,7 +12054,7 @@
         <v>296</v>
       </c>
       <c r="F61" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G61">
         <v>4</v>
@@ -12031,7 +12089,7 @@
     </row>
     <row r="62" spans="1:16">
       <c r="A62" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B62">
         <v>6926834</v>
@@ -12073,7 +12131,7 @@
         <v>45512</v>
       </c>
       <c r="O62" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P62">
         <v>2520</v>
@@ -12896,7 +12954,7 @@
         <v>298</v>
       </c>
       <c r="F79" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G79">
         <v>5</v>
@@ -13287,7 +13345,7 @@
         <v>7266797</v>
       </c>
       <c r="C87" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D87" t="s">
         <v>284</v>
@@ -13323,7 +13381,7 @@
         <v>45523</v>
       </c>
       <c r="O87" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="P87">
         <v>21700</v>
@@ -13481,7 +13539,7 @@
     </row>
     <row r="91" spans="1:16">
       <c r="A91" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B91">
         <v>9247453</v>
@@ -13523,7 +13581,7 @@
         <v>45583</v>
       </c>
       <c r="O91" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P91">
         <v>3240</v>
@@ -13946,7 +14004,7 @@
         <v>305</v>
       </c>
       <c r="F100" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G100">
         <v>297</v>
@@ -14946,7 +15004,7 @@
         <v>310</v>
       </c>
       <c r="F120" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G120">
         <v>100</v>
@@ -15537,7 +15595,7 @@
         <v>649634</v>
       </c>
       <c r="C132" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D132" t="s">
         <v>285</v>
@@ -15573,7 +15631,7 @@
         <v>45674</v>
       </c>
       <c r="O132" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="P132">
         <v>18400</v>
@@ -15881,7 +15939,7 @@
     </row>
     <row r="139" spans="1:16">
       <c r="A139" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B139">
         <v>3333331</v>
@@ -15923,7 +15981,7 @@
         <v>45755</v>
       </c>
       <c r="O139" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P139">
         <v>3700</v>
@@ -16046,7 +16104,7 @@
         <v>312</v>
       </c>
       <c r="F142" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G142">
         <v>33</v>
@@ -16431,7 +16489,7 @@
     </row>
     <row r="150" spans="1:16">
       <c r="A150" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B150">
         <v>6004728</v>
@@ -16473,7 +16531,7 @@
         <v>45849</v>
       </c>
       <c r="O150" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P150">
         <v>3520</v>
@@ -16481,7 +16539,7 @@
     </row>
     <row r="151" spans="1:16">
       <c r="A151" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B151">
         <v>6004729</v>
@@ -16523,7 +16581,7 @@
         <v>45849</v>
       </c>
       <c r="O151" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P151">
         <v>2.79</v>
@@ -16581,7 +16639,7 @@
     </row>
     <row r="153" spans="1:16">
       <c r="A153" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B153">
         <v>6069005</v>
@@ -16623,7 +16681,7 @@
         <v>45852</v>
       </c>
       <c r="O153" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="P153">
         <v>3695.1428571428</v>
@@ -19046,7 +19104,7 @@
         <v>328</v>
       </c>
       <c r="F202" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G202">
         <v>90</v>
@@ -19846,7 +19904,7 @@
         <v>337</v>
       </c>
       <c r="F218" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G218">
         <v>100</v>
@@ -19887,7 +19945,7 @@
         <v>10583557</v>
       </c>
       <c r="C219" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D219" t="s">
         <v>284</v>
@@ -19923,7 +19981,7 @@
         <v>46283</v>
       </c>
       <c r="O219" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="P219">
         <v>23880</v>
@@ -19946,7 +20004,7 @@
         <v>339</v>
       </c>
       <c r="F220" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="G220">
         <v>232</v>
@@ -20027,6 +20085,56 @@
       </c>
       <c r="P221">
         <v>15134.9640287769</v>
+      </c>
+    </row>
+    <row r="222" spans="1:16">
+      <c r="A222" t="s">
+        <v>200</v>
+      </c>
+      <c r="B222">
+        <v>10845350</v>
+      </c>
+      <c r="C222" t="s">
+        <v>269</v>
+      </c>
+      <c r="D222" t="s">
+        <v>284</v>
+      </c>
+      <c r="E222" t="s">
+        <v>340</v>
+      </c>
+      <c r="F222" t="s">
+        <v>355</v>
+      </c>
+      <c r="G222">
+        <v>195</v>
+      </c>
+      <c r="H222">
+        <v>5110</v>
+      </c>
+      <c r="I222">
+        <v>996450</v>
+      </c>
+      <c r="J222">
+        <v>602.85</v>
+      </c>
+      <c r="K222">
+        <v>6028.52</v>
+      </c>
+      <c r="L222">
+        <v>1003081.37</v>
+      </c>
+      <c r="M222" t="s">
+        <v>190</v>
+      </c>
+      <c r="N222" s="1">
+        <v>46289</v>
+      </c>
+      <c r="O222" t="s">
+        <v>200</v>
+      </c>
+      <c r="P222">
+        <v>5110</v>
       </c>
     </row>
   </sheetData>
@@ -20049,15 +20157,15 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B2">
-        <v>2113593.05</v>
+        <v>1110511.68</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B3">
         <v>1292494.146087911</v>
@@ -20065,10 +20173,10 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B4">
-        <v>2217162.070769231</v>
+        <v>1167749.330769231</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🤖 Motor ejecutado: Cálculos actualizados
</commit_message>
<xml_diff>
--- a/mi_cartera_balanz/data/Reporte_Avanzado_Cartera.xlsx
+++ b/mi_cartera_balanz/data/Reporte_Avanzado_Cartera.xlsx
@@ -329,8 +329,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -346,7 +354,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -354,12 +362,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,31 +685,31 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1335,28 +1361,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
     </row>
@@ -1377,13 +1403,13 @@
         <v>34</v>
       </c>
       <c r="F2">
-        <v>9670</v>
+        <v>9675</v>
       </c>
       <c r="G2">
-        <v>58020</v>
+        <v>58050</v>
       </c>
       <c r="H2">
-        <v>20548.67</v>
+        <v>20578.67</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1403,13 +1429,13 @@
         <v>34</v>
       </c>
       <c r="F3">
-        <v>16220</v>
+        <v>16100</v>
       </c>
       <c r="G3">
-        <v>5320160</v>
+        <v>5280800</v>
       </c>
       <c r="H3">
-        <v>1699442.89</v>
+        <v>1660082.89</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1429,13 +1455,13 @@
         <v>34</v>
       </c>
       <c r="F4">
-        <v>8225</v>
+        <v>8190</v>
       </c>
       <c r="G4">
-        <v>995225</v>
+        <v>990990</v>
       </c>
       <c r="H4">
-        <v>3730.219999999856</v>
+        <v>-504.7800000001444</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1527,36 +1553,36 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="1">
+      <c r="A2" s="2">
         <v>45588</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>45667</v>
       </c>
       <c r="C2" t="s">
@@ -1579,10 +1605,10 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="1">
+      <c r="A3" s="2">
         <v>45588</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>45922</v>
       </c>
       <c r="C3" t="s">
@@ -1605,10 +1631,10 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="1">
+      <c r="A4" s="2">
         <v>45623</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>45922</v>
       </c>
       <c r="C4" t="s">
@@ -1631,10 +1657,10 @@
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="1">
+      <c r="A5" s="2">
         <v>45656</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="2">
         <v>45922</v>
       </c>
       <c r="C5" t="s">
@@ -1657,10 +1683,10 @@
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="1">
+      <c r="A6" s="2">
         <v>45667</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="2">
         <v>45922</v>
       </c>
       <c r="C6" t="s">
@@ -1683,10 +1709,10 @@
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="1">
+      <c r="A7" s="2">
         <v>45667</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="2">
         <v>45922</v>
       </c>
       <c r="C7" t="s">
@@ -1709,10 +1735,10 @@
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="1">
+      <c r="A8" s="2">
         <v>45852</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="2">
         <v>45922</v>
       </c>
       <c r="C8" t="s">
@@ -1745,28 +1771,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1774,7 +1800,7 @@
       <c r="A2" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="2">
         <v>45922</v>
       </c>
       <c r="C2">
@@ -1800,7 +1826,7 @@
       <c r="A3" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="2">
         <v>45922</v>
       </c>
       <c r="C3">
@@ -1826,7 +1852,7 @@
       <c r="A4" t="s">
         <v>44</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="2">
         <v>46294</v>
       </c>
       <c r="C4">
@@ -1859,10 +1885,10 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1973,52 +1999,52 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>85</v>
       </c>
     </row>
@@ -2062,7 +2088,7 @@
       <c r="M2" t="s">
         <v>34</v>
       </c>
-      <c r="N2" s="1">
+      <c r="N2" s="2">
         <v>45588</v>
       </c>
       <c r="O2" t="s">
@@ -2112,7 +2138,7 @@
       <c r="M3" t="s">
         <v>34</v>
       </c>
-      <c r="N3" s="1">
+      <c r="N3" s="2">
         <v>45623</v>
       </c>
       <c r="O3" t="s">
@@ -2162,7 +2188,7 @@
       <c r="M4" t="s">
         <v>34</v>
       </c>
-      <c r="N4" s="1">
+      <c r="N4" s="2">
         <v>45656</v>
       </c>
       <c r="O4" t="s">
@@ -2212,7 +2238,7 @@
       <c r="M5" t="s">
         <v>34</v>
       </c>
-      <c r="N5" s="1">
+      <c r="N5" s="2">
         <v>45667</v>
       </c>
       <c r="O5" t="s">
@@ -2262,7 +2288,7 @@
       <c r="M6" t="s">
         <v>36</v>
       </c>
-      <c r="N6" s="1">
+      <c r="N6" s="2">
         <v>45667</v>
       </c>
       <c r="O6" t="s">
@@ -2312,7 +2338,7 @@
       <c r="M7" t="s">
         <v>34</v>
       </c>
-      <c r="N7" s="1">
+      <c r="N7" s="2">
         <v>45667</v>
       </c>
       <c r="O7" t="s">
@@ -2362,7 +2388,7 @@
       <c r="M8" t="s">
         <v>36</v>
       </c>
-      <c r="N8" s="1">
+      <c r="N8" s="2">
         <v>45852</v>
       </c>
       <c r="O8" t="s">
@@ -2412,7 +2438,7 @@
       <c r="M9" t="s">
         <v>34</v>
       </c>
-      <c r="N9" s="1">
+      <c r="N9" s="2">
         <v>45922</v>
       </c>
       <c r="O9" t="s">
@@ -2462,7 +2488,7 @@
       <c r="M10" t="s">
         <v>34</v>
       </c>
-      <c r="N10" s="1">
+      <c r="N10" s="2">
         <v>45922</v>
       </c>
       <c r="O10" t="s">
@@ -2512,7 +2538,7 @@
       <c r="M11" t="s">
         <v>34</v>
       </c>
-      <c r="N11" s="1">
+      <c r="N11" s="2">
         <v>45922</v>
       </c>
       <c r="O11" t="s">
@@ -2562,7 +2588,7 @@
       <c r="M12" t="s">
         <v>34</v>
       </c>
-      <c r="N12" s="1">
+      <c r="N12" s="2">
         <v>46294</v>
       </c>
       <c r="O12" t="s">
@@ -2583,10 +2609,10 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>63</v>
       </c>
     </row>
@@ -2611,7 +2637,7 @@
         <v>99</v>
       </c>
       <c r="B4">
-        <v>1723716.69</v>
+        <v>1680151.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>